<commit_message>
feat(path): add the adult chapters (Ch.6–8) from the updated master node table
The Master Node Table now covers the full lifelong path: kids Ch.1–5 plus the
adult journey — Ch.6 College (18–22), Ch.7 Building a Life (22 → first child),
Ch.8 Parenthood + Parent Layer. Regenerate path.ts from it:

- Sync scripts/master-node-table.xlsx with the updated 79-row table.
- gen-path.py: add fitting emoji for the 29 adult nodes (g44–g69, c6–c8) and
  subtitles for Ch.6/7/8; widen ThreadKey for the new compound threads D/E & F/D
  and tag D/E as a gender node.
- Regenerate: NODES now 77 (was 48), CHAPTERS 8 (was 5). The adult games aren't
  built yet, so those nodes render as the disabled "soon" treatment — same as the
  unbuilt kids games.

Canvas myth/doodle dressing for Ch.6–8 is a separate follow-up (it comes from the
adult GDD myth banks, not the node table).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/master-node-table.xlsx
+++ b/scripts/master-node-table.xlsx
@@ -92,7 +92,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -169,6 +169,11 @@
         <fgColor rgb="FFF8CBAD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -196,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -306,6 +311,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -671,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:N79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -693,7 +701,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SwipeEd — Master Node Table  (drop-in path spec: 43 games + 5 capstones, in order)</t>
+          <t>SwipeEd — Master Node Table  (full lifelong path: kids' Ch.1–5 + adult Ch.6 College · Ch.7 Building a Life · Ch.8 Parenthood + Parent Layer)</t>
         </is>
       </c>
     </row>
@@ -4028,6 +4036,1978 @@
         </is>
       </c>
       <c r="N50" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>g44</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Consent, For Real</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Ch.6 · Ages 18–22</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G51" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>Safety, Consent &amp; Boundaries</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t>#DC2626</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>4.2, 4.1, 5.5</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>c5</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>g31</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>Adult consent in practice: alcohol, an ongoing yes, assault awareness &amp; survivor support</t>
+        </is>
+      </c>
+      <c r="N51" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>g45</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Swipe Right? — Dating &amp; Apps</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Ch.6 · Ages 18–22</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Relationships</t>
+        </is>
+      </c>
+      <c r="I52" s="7" t="inlineStr">
+        <is>
+          <t>#EC4899</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>1.2, 4.3, 5.5</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>g44</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>g24</t>
+        </is>
+      </c>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>Modern dating &amp; app safety: meeting safely, ghosting, catfishing, digital boundaries</t>
+        </is>
+      </c>
+      <c r="N52" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>g46</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Real Relationships</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Ch.6 · Ages 18–22</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Relationships</t>
+        </is>
+      </c>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>#EC4899</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>1.2, 5.3, 4.1, 5.6</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>g45</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>g31</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>Building healthy adult relationships; recognising &amp; leaving unhealthy ones; breakups</t>
+        </is>
+      </c>
+      <c r="N53" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>g47</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Own Your Health</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Ch.6 · Ages 18–22</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G54" s="18" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>Sexual &amp; Reproductive Health</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>#059669</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>8.1, 8.2, 8.3, 7.2</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>g46</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>g30</t>
+        </is>
+      </c>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>Adult SRH ownership: contraception, routine testing, sexual wellbeing &amp; pleasure, services</t>
+        </is>
+      </c>
+      <c r="N54" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>g48</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Money &amp; Independence</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Ch.6 · Ages 18–22</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>Feelings &amp; Life Skills</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>#F59E0B</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>5.2, 2.2</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>g47</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>g42</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>Work &amp; money: financial literacy &amp; independence; money in relationships</t>
+        </is>
+      </c>
+      <c r="N55" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>g49</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Mind &amp; Belonging</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Ch.6 · Ages 18–22</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>Feelings &amp; Life Skills</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>#F59E0B</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>5.6, 5.5, 6.4</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>g48</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>g39</t>
+        </is>
+      </c>
+      <c r="M56" s="5" t="inlineStr">
+        <is>
+          <t>College mental health, loneliness &amp; leaving home; body image; help-seeking</t>
+        </is>
+      </c>
+      <c r="N56" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>g52</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Find Your Feet</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Ch.6 · Ages 18–22</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>Feelings &amp; Life Skills</t>
+        </is>
+      </c>
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t>#F59E0B</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>5.6, 5.2, 5.1, 5.5</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>g49</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>g42</t>
+        </is>
+      </c>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>Career &amp; future anxiety: comparison, the pressure to have it ‘figured out’, purpose &amp; worth beyond your CV</t>
+        </is>
+      </c>
+      <c r="N57" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>g50</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Equal &amp; Confident</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Ch.6 · Ages 18–22</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G58" s="10" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>Gender &amp; Respect</t>
+        </is>
+      </c>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t>#7C3AED</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>3.2, 3.1</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>g52</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>g33</t>
+        </is>
+      </c>
+      <c r="M58" s="5" t="inlineStr">
+        <is>
+          <t>Gender equality at college/work; allyship; confidence, voice &amp; leadership</t>
+        </is>
+      </c>
+      <c r="N58" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>g51</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Know Your Rights (Adult)</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Ch.6 · Ages 18–22</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G59" s="17" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>Values, Rights &amp; Media</t>
+        </is>
+      </c>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>#475569</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>2.2, 4.3, 3.3</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>g50</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>g35</t>
+        </is>
+      </c>
+      <c r="M59" s="5" t="inlineStr">
+        <is>
+          <t>Adult rights: POSH/harassment, consent law, work/tenancy/cyber rights</t>
+        </is>
+      </c>
+      <c r="N59" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>c6</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>Capstone: Standing on My Own</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Capstone</t>
+        </is>
+      </c>
+      <c r="E60" s="13" t="inlineStr">
+        <is>
+          <t>Ch.6 · Ages 18–22</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="G60" s="14" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="H60" s="13" t="inlineStr">
+        <is>
+          <t>Capstone milestone</t>
+        </is>
+      </c>
+      <c r="I60" s="15" t="inlineStr">
+        <is>
+          <t>#EAB308</t>
+        </is>
+      </c>
+      <c r="J60" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K60" s="11" t="inlineStr">
+        <is>
+          <t>g51</t>
+        </is>
+      </c>
+      <c r="L60" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M60" s="13" t="inlineStr">
+        <is>
+          <t>Chapter 6 graduation — an independent young adult</t>
+        </is>
+      </c>
+      <c r="N60" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>g53</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Choosing &amp; Building</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Ch.7 · 22 → first child</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G61" s="9" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>Relationships</t>
+        </is>
+      </c>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>#EC4899</t>
+        </is>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>1.2, 1.4, 5.3, 2.1</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>c6</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>g46</t>
+        </is>
+      </c>
+      <c r="M61" s="5" t="inlineStr">
+        <is>
+          <t>Choosing a partner &amp; what makes a healthy long-term partnership/marriage (love &amp; arranged); commitment &amp; communication</t>
+        </is>
+      </c>
+      <c r="N61" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>g54</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Your Path, Your Call</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Ch.7 · 22 → first child</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G62" s="9" t="inlineStr">
+        <is>
+          <t>D/E</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>Relationships · Gender</t>
+        </is>
+      </c>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>#EC4899</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>1.2, 3.2, 2.2, 5.2</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>g53</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>g50</t>
+        </is>
+      </c>
+      <c r="M62" s="5" t="inlineStr">
+        <is>
+          <t>The freedom not to marry or have children; resisting the ‘settle down’ / ‘still-unmarried’ pressure (esp. on women); worth beyond marital status &amp; looks</t>
+        </is>
+      </c>
+      <c r="N62" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>g55</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Equal Partners</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Ch.7 · 22 → first child</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G63" s="10" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>Gender &amp; Respect</t>
+        </is>
+      </c>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>#7C3AED</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>3.2, 1.1, 5.3</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>g54</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>g26</t>
+        </is>
+      </c>
+      <c r="M63" s="5" t="inlineStr">
+        <is>
+          <t>The equal home: sharing the domestic &amp; care load (the second shift), dual careers, equality in the relationship</t>
+        </is>
+      </c>
+      <c r="N63" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>g56</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Respect at Home</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Ch.7 · 22 → first child</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G64" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>Safety, Consent &amp; Boundaries</t>
+        </is>
+      </c>
+      <c r="I64" s="7" t="inlineStr">
+        <is>
+          <t>#DC2626</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>4.2, 4.1, 5.5</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>g55</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>g31</t>
+        </is>
+      </c>
+      <c r="M64" s="5" t="inlineStr">
+        <is>
+          <t>Consent &amp; mutual respect in marriage; recognising &amp; responding to coercion/DV; where to get help</t>
+        </is>
+      </c>
+      <c r="N64" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>g57</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>The Family Map</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Ch.7 · 22 → first child</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G65" s="9" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>Relationships</t>
+        </is>
+      </c>
+      <c r="I65" s="7" t="inlineStr">
+        <is>
+          <t>#EC4899</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>1.1, 2.3, 5.3</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>g56</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>g03</t>
+        </is>
+      </c>
+      <c r="M65" s="5" t="inlineStr">
+        <is>
+          <t>In-laws &amp; extended/joint family: navigating dynamics, setting boundaries, finding your place</t>
+        </is>
+      </c>
+      <c r="N65" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>g58</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Money, Together</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Ch.7 · 22 → first child</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>Feelings &amp; Life Skills</t>
+        </is>
+      </c>
+      <c r="I66" s="7" t="inlineStr">
+        <is>
+          <t>#F59E0B</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>5.2, 2.2</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>g57</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>g48</t>
+        </is>
+      </c>
+      <c r="M66" s="5" t="inlineStr">
+        <is>
+          <t>Work &amp; money: joint finances &amp; planning; financial independence within a partnership; financial control as abuse</t>
+        </is>
+      </c>
+      <c r="N66" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>g59</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>If, When &amp; Whether</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Ch.7 · 22 → first child</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G67" s="18" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>Sexual &amp; Reproductive Health</t>
+        </is>
+      </c>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>#059669</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>8.1, 6.2, 6.3</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>g58</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>g29</t>
+        </is>
+      </c>
+      <c r="M67" s="5" t="inlineStr">
+        <is>
+          <t>Reproductive planning: whether, when &amp; spacing children; fertility awareness; preconception health; infertility &amp; options</t>
+        </is>
+      </c>
+      <c r="N67" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>g60</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Many Ways to Family</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Ch.7 · 22 → first child</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G68" s="18" t="inlineStr">
+        <is>
+          <t>F/D</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>SRH · Relationships</t>
+        </is>
+      </c>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t>#059669</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>8.1, 1.1, 2.2</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>g59</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>g32</t>
+        </is>
+      </c>
+      <c r="M68" s="5" t="inlineStr">
+        <is>
+          <t>Diverse routes to family — adoption/fostering, surrogacy &amp; IVF, single &amp; LGBTQ+ parenthood — and the gendered barriers (e.g. single men &amp; girl-child adoption, CARA 2022)</t>
+        </is>
+      </c>
+      <c r="N68" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>c7</t>
+        </is>
+      </c>
+      <c r="C69" s="12" t="inlineStr">
+        <is>
+          <t>Capstone: Building Together</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
+        <is>
+          <t>Capstone</t>
+        </is>
+      </c>
+      <c r="E69" s="13" t="inlineStr">
+        <is>
+          <t>Ch.7 · 22 → first child</t>
+        </is>
+      </c>
+      <c r="F69" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="G69" s="14" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="H69" s="13" t="inlineStr">
+        <is>
+          <t>Capstone milestone</t>
+        </is>
+      </c>
+      <c r="I69" s="15" t="inlineStr">
+        <is>
+          <t>#EAB308</t>
+        </is>
+      </c>
+      <c r="J69" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K69" s="11" t="inlineStr">
+        <is>
+          <t>g60</t>
+        </is>
+      </c>
+      <c r="L69" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M69" s="13" t="inlineStr">
+        <is>
+          <t>Chapter 7 graduation — a life built together, or on your own terms</t>
+        </is>
+      </c>
+      <c r="N69" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>g61</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Us, After Kids</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Ch.8 · Parenthood (first child on)</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>Relationships</t>
+        </is>
+      </c>
+      <c r="I70" s="7" t="inlineStr">
+        <is>
+          <t>#EC4899</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>1.2, 5.3, 7.1</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>c7</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>g53</t>
+        </is>
+      </c>
+      <c r="M70" s="5" t="inlineStr">
+        <is>
+          <t>Keeping the partnership &amp; intimacy alive with kids in the picture; co-parenting connection &amp; communication under load</t>
+        </is>
+      </c>
+      <c r="N70" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>g62</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Equal Parents</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Ch.8 · Parenthood (first child on)</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G71" s="10" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>Gender &amp; Respect</t>
+        </is>
+      </c>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>#7C3AED</t>
+        </is>
+      </c>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>3.2, 1.4, 1.1</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>g61</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>g55</t>
+        </is>
+      </c>
+      <c r="M71" s="5" t="inlineStr">
+        <is>
+          <t>Co-parenting as equals — sharing the care &amp; mental load, involved fatherhood, breaking gendered parenting</t>
+        </is>
+      </c>
+      <c r="N71" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>g63</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Looking After You</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Ch.8 · Parenthood (first child on)</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>Feelings &amp; Life Skills</t>
+        </is>
+      </c>
+      <c r="I72" s="7" t="inlineStr">
+        <is>
+          <t>#F59E0B</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>5.6, 5.5</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>g62</t>
+        </is>
+      </c>
+      <c r="L72" s="3" t="inlineStr">
+        <is>
+          <t>g49</t>
+        </is>
+      </c>
+      <c r="M72" s="5" t="inlineStr">
+        <is>
+          <t>Parental wellbeing &amp; mental health; burnout; your own needs matter; the Life-Skills Toolkit under load</t>
+        </is>
+      </c>
+      <c r="N72" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>g64</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>The Talks (Age by Age)</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Ch.8 · Parenthood (first child on)</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G73" s="18" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>Parent Layer · RSE guidance</t>
+        </is>
+      </c>
+      <c r="I73" s="7" t="inlineStr">
+        <is>
+          <t>#059669</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>4.2, 6.3, 7.1, 2.1</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>g63</t>
+        </is>
+      </c>
+      <c r="L73" s="3" t="inlineStr">
+        <is>
+          <t>g02</t>
+        </is>
+      </c>
+      <c r="M73" s="5" t="inlineStr">
+        <is>
+          <t>PARENT LAYER — age-by-age RSE guidance mapped to your child's journey (bodies, consent, puberty, relationships, sexuality, online); many small talks; facts + your values</t>
+        </is>
+      </c>
+      <c r="N73" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>g65</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Break the Cycle</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Ch.8 · Parenthood (first child on)</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>Parent Layer · Positive Parenting</t>
+        </is>
+      </c>
+      <c r="I74" s="7" t="inlineStr">
+        <is>
+          <t>#F59E0B</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>5.6, 5.3</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>g64</t>
+        </is>
+      </c>
+      <c r="L74" s="3" t="inlineStr">
+        <is>
+          <t>g38</t>
+        </is>
+      </c>
+      <c r="M74" s="5" t="inlineStr">
+        <is>
+          <t>Positive parenting &amp; breaking generational trauma; discipline without fear, shame or hitting; repair; healing your own wounds (Unlearn→Relearn, for parents)</t>
+        </is>
+      </c>
+      <c r="N74" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>g66</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>Raising Gender-Diverse Kids</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Ch.8 · Parenthood (first child on)</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G75" s="10" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>Parent Layer · Positive Parenting</t>
+        </is>
+      </c>
+      <c r="I75" s="7" t="inlineStr">
+        <is>
+          <t>#7C3AED</t>
+        </is>
+      </c>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>3.1, 1.3, 7.1</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>g65</t>
+        </is>
+      </c>
+      <c r="L75" s="3" t="inlineStr">
+        <is>
+          <t>g32</t>
+        </is>
+      </c>
+      <c r="M75" s="5" t="inlineStr">
+        <is>
+          <t>Affirming &amp; protecting an LGBTQ+ or gender-nonconforming child; not forcing norms; being their safe place</t>
+        </is>
+      </c>
+      <c r="N75" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>g67</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Raising Neurodiverse Kids</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Ch.8 · Parenthood (first child on)</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>Parent Layer · Positive Parenting</t>
+        </is>
+      </c>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>#F59E0B</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>5.6, 1.3, 5.5</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>g66</t>
+        </is>
+      </c>
+      <c r="L76" s="3" t="inlineStr">
+        <is>
+          <t>g04</t>
+        </is>
+      </c>
+      <c r="M76" s="5" t="inlineStr">
+        <is>
+          <t>Understanding &amp; supporting autism, ADHD &amp; learning differences; accommodating, advocating, de-stigmatising</t>
+        </is>
+      </c>
+      <c r="N76" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>g68</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Navigating Addictions</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Ch.8 · Parenthood (first child on)</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G77" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>Parent Layer · Positive Parenting</t>
+        </is>
+      </c>
+      <c r="I77" s="7" t="inlineStr">
+        <is>
+          <t>#DC2626</t>
+        </is>
+      </c>
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>5.1, 5.5, 5.6</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>g67</t>
+        </is>
+      </c>
+      <c r="L77" s="3" t="inlineStr">
+        <is>
+          <t>g39</t>
+        </is>
+      </c>
+      <c r="M77" s="5" t="inlineStr">
+        <is>
+          <t>Recognising &amp; responding (without shame) to a child's substance / screen / gaming dependence; getting help early; modelling healthy habits</t>
+        </is>
+      </c>
+      <c r="N77" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>g69</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Be the Safe Adult</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Ch.8 · Parenthood (first child on)</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G78" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>Parent Layer · Safeguarding</t>
+        </is>
+      </c>
+      <c r="I78" s="7" t="inlineStr">
+        <is>
+          <t>#DC2626</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>4.1, 4.2, 4.3, 5.5</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>g68</t>
+        </is>
+      </c>
+      <c r="L78" s="3" t="inlineStr">
+        <is>
+          <t>g08</t>
+        </is>
+      </c>
+      <c r="M78" s="5" t="inlineStr">
+        <is>
+          <t>Safeguarding literacy: spotting abuse, POCSO basics, online dangers, and how to respond to a disclosure — the trusted adult the kids' journey assumes</t>
+        </is>
+      </c>
+      <c r="N78" s="39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="n">
+        <v>77</v>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>c8</t>
+        </is>
+      </c>
+      <c r="C79" s="12" t="inlineStr">
+        <is>
+          <t>Capstone: Raising the Next Generation</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>Capstone</t>
+        </is>
+      </c>
+      <c r="E79" s="13" t="inlineStr">
+        <is>
+          <t>Ch.8 · Parenthood (first child on)</t>
+        </is>
+      </c>
+      <c r="F79" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="G79" s="14" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="H79" s="13" t="inlineStr">
+        <is>
+          <t>Capstone milestone</t>
+        </is>
+      </c>
+      <c r="I79" s="15" t="inlineStr">
+        <is>
+          <t>#EAB308</t>
+        </is>
+      </c>
+      <c r="J79" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K79" s="11" t="inlineStr">
+        <is>
+          <t>g69</t>
+        </is>
+      </c>
+      <c r="L79" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M79" s="13" t="inlineStr">
+        <is>
+          <t>Final graduation — guiding the next generation; the loop comes full circle</t>
+        </is>
+      </c>
+      <c r="N79" s="32" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4047,7 +6027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4420,6 +6400,48 @@
       <c r="A37" s="36" t="inlineStr">
         <is>
           <t>Added g43 The Rabbit Hole (online misogyny &amp; the manosphere; Ch.4; dual thread E/G, node colour slate; topics 3.2/3.1/5.4/5.1/1.3; gating Gated) after g40 Firewall. Non-shaming, positive-masculinity-centred. Now 43 games + 5 capstones = 48 nodes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="38" t="inlineStr">
+        <is>
+          <t>Adult journey — Ch.6 College added (June 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="36" t="inlineStr">
+        <is>
+          <t>Adult chapters continue the same product &amp; linear chain. Ch.6 College (18–22): g44–g52 + c6. gating ‘Open’ = adult, comprehensive, not school-comfort-gated. Chapters 7 (Building a Life) &amp; 8 (Parenthood + Parent Layer) to follow, one layer at a time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="38" t="inlineStr">
+        <is>
+          <t>Adult journey — Ch.7 Building a Life added (June 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="36" t="inlineStr">
+        <is>
+          <t>Ch.7 (22 → first child): g53–g60 + c7. Includes the diverse-paths content — freedom not to marry/childfree &amp; the ‘still-unmarried’ stigma (g54), and diverse routes to family incl. the single-man / girl-child adoption barrier (g60). Ch.8 Parenthood + the Parent Layer to follow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="38" t="inlineStr">
+        <is>
+          <t>Adult journey — Ch.8 Parenthood + Parent Layer added (June 2026); adult node-map complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="36" t="inlineStr">
+        <is>
+          <t>Ch.8 (first child on): g61–g63 = the parent's own continuing journey; g64–g69 = the PARENT LAYER (‘SwipeEd Raising’) — age-by-age RSE guidance (g64) + positive parenting: break the cycle/generational trauma (g65), raising gender-diverse (g66) &amp; neurodiverse (g67) kids, navigating addictions (g68), being the safe adult (g69). c8 closes the generational loop. The full lifelong journey (Ch.1–8) is now mapped.</t>
         </is>
       </c>
     </row>

</xml_diff>